<commit_message>
re-align the rolling cnt, re-query, re-script, re-compilation
</commit_message>
<xml_diff>
--- a/data/Simulation_User_Summary.xlsx
+++ b/data/Simulation_User_Summary.xlsx
@@ -5,19 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wei.kc\Desktop\Adhoc\03 Sept 2026\data\VN_order(July-Aug)\Compiled_Output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wei.kc\Desktop\Adhoc\03 Sept 2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{306ADA99-4FC0-4367-B52B-E9FF525C8CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD14C98E-C8D4-4114-A213-EF76DD6EC84D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="user-summary (July_Aug2026)" sheetId="1" r:id="rId1"/>
-    <sheet name="linkage" sheetId="2" r:id="rId2"/>
+    <sheet name="user-summary(July2026)" sheetId="3" r:id="rId2"/>
+    <sheet name="user-summary(Aug2026)" sheetId="4" r:id="rId3"/>
+    <sheet name="linkage" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">linkage!$A$1:$C$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">linkage!$A$1:$C$52</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="119">
   <si>
     <t>user_id</t>
   </si>
@@ -252,12 +254,6 @@
     <t>51.74%</t>
   </si>
   <si>
-    <t>19.87%</t>
-  </si>
-  <si>
-    <t>49.7%</t>
-  </si>
-  <si>
     <t>70.0%</t>
   </si>
   <si>
@@ -397,6 +393,12 @@
   </si>
   <si>
     <t>Count</t>
+  </si>
+  <si>
+    <t>19.83%</t>
+  </si>
+  <si>
+    <t>49.81%</t>
   </si>
 </sst>
 </file>
@@ -822,7 +824,7 @@
         <v>15</v>
       </c>
       <c r="J2">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="K2">
         <v>37</v>
@@ -869,7 +871,7 @@
         <v>18</v>
       </c>
       <c r="J3">
-        <v>92</v>
+        <v>58</v>
       </c>
       <c r="K3">
         <v>115</v>
@@ -916,7 +918,7 @@
         <v>21</v>
       </c>
       <c r="J4">
-        <v>221</v>
+        <v>66</v>
       </c>
       <c r="K4">
         <v>262</v>
@@ -963,7 +965,7 @@
         <v>23</v>
       </c>
       <c r="J5">
-        <v>165</v>
+        <v>70</v>
       </c>
       <c r="K5">
         <v>204</v>
@@ -1010,7 +1012,7 @@
         <v>25</v>
       </c>
       <c r="J6">
-        <v>191</v>
+        <v>125</v>
       </c>
       <c r="K6">
         <v>215</v>
@@ -1057,7 +1059,7 @@
         <v>27</v>
       </c>
       <c r="J7">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="K7">
         <v>26</v>
@@ -1104,7 +1106,7 @@
         <v>29</v>
       </c>
       <c r="J8">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="K8">
         <v>23</v>
@@ -1151,7 +1153,7 @@
         <v>31</v>
       </c>
       <c r="J9">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="K9">
         <v>49</v>
@@ -1198,7 +1200,7 @@
         <v>33</v>
       </c>
       <c r="J10">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="K10">
         <v>68</v>
@@ -1245,7 +1247,7 @@
         <v>35</v>
       </c>
       <c r="J11">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="K11">
         <v>26</v>
@@ -1292,7 +1294,7 @@
         <v>37</v>
       </c>
       <c r="J12">
-        <v>308</v>
+        <v>103</v>
       </c>
       <c r="K12">
         <v>353</v>
@@ -1339,7 +1341,7 @@
         <v>39</v>
       </c>
       <c r="J13">
-        <v>215</v>
+        <v>100</v>
       </c>
       <c r="K13">
         <v>228</v>
@@ -1386,7 +1388,7 @@
         <v>41</v>
       </c>
       <c r="J14">
-        <v>162</v>
+        <v>65</v>
       </c>
       <c r="K14">
         <v>195</v>
@@ -1433,7 +1435,7 @@
         <v>44</v>
       </c>
       <c r="J15">
-        <v>193</v>
+        <v>99</v>
       </c>
       <c r="K15">
         <v>201</v>
@@ -1480,7 +1482,7 @@
         <v>47</v>
       </c>
       <c r="J16">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="K16">
         <v>196</v>
@@ -1527,7 +1529,7 @@
         <v>50</v>
       </c>
       <c r="J17">
-        <v>125</v>
+        <v>97</v>
       </c>
       <c r="K17">
         <v>132</v>
@@ -1574,7 +1576,7 @@
         <v>53</v>
       </c>
       <c r="J18">
-        <v>185</v>
+        <v>97</v>
       </c>
       <c r="K18">
         <v>197</v>
@@ -1621,7 +1623,7 @@
         <v>55</v>
       </c>
       <c r="J19">
-        <v>137</v>
+        <v>109</v>
       </c>
       <c r="K19">
         <v>165</v>
@@ -1668,7 +1670,7 @@
         <v>58</v>
       </c>
       <c r="J20">
-        <v>101</v>
+        <v>66</v>
       </c>
       <c r="K20">
         <v>134</v>
@@ -1715,7 +1717,7 @@
         <v>61</v>
       </c>
       <c r="J21">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="K21">
         <v>119</v>
@@ -1762,7 +1764,7 @@
         <v>64</v>
       </c>
       <c r="J22">
-        <v>131</v>
+        <v>76</v>
       </c>
       <c r="K22">
         <v>155</v>
@@ -1809,7 +1811,7 @@
         <v>66</v>
       </c>
       <c r="J23">
-        <v>146</v>
+        <v>81</v>
       </c>
       <c r="K23">
         <v>168</v>
@@ -1856,22 +1858,22 @@
         <v>69</v>
       </c>
       <c r="J24">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="K24">
-        <v>4107</v>
+        <v>4116</v>
       </c>
       <c r="L24">
         <v>816</v>
       </c>
       <c r="M24">
-        <v>2041</v>
+        <v>2050</v>
       </c>
       <c r="N24" t="s">
-        <v>70</v>
+        <v>117</v>
       </c>
       <c r="O24" t="s">
-        <v>71</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
@@ -1900,10 +1902,10 @@
         <v>130</v>
       </c>
       <c r="I25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J25">
-        <v>107</v>
+        <v>77</v>
       </c>
       <c r="K25">
         <v>130</v>
@@ -1918,7 +1920,7 @@
         <v>19</v>
       </c>
       <c r="O25" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
@@ -1947,10 +1949,10 @@
         <v>133</v>
       </c>
       <c r="I26" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J26">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="K26">
         <v>133</v>
@@ -1965,7 +1967,7 @@
         <v>59</v>
       </c>
       <c r="O26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
@@ -1994,10 +1996,10 @@
         <v>101</v>
       </c>
       <c r="I27" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J27">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="K27">
         <v>101</v>
@@ -2012,7 +2014,7 @@
         <v>19</v>
       </c>
       <c r="O27" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
@@ -2041,10 +2043,10 @@
         <v>126</v>
       </c>
       <c r="I28" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J28">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="K28">
         <v>126</v>
@@ -2059,7 +2061,7 @@
         <v>19</v>
       </c>
       <c r="O28" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
@@ -2088,10 +2090,10 @@
         <v>80</v>
       </c>
       <c r="I29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="J29">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="K29">
         <v>80</v>
@@ -2106,7 +2108,7 @@
         <v>19</v>
       </c>
       <c r="O29" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
@@ -2135,10 +2137,10 @@
         <v>130</v>
       </c>
       <c r="I30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J30">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="K30">
         <v>130</v>
@@ -2153,7 +2155,7 @@
         <v>28</v>
       </c>
       <c r="O30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
@@ -2182,10 +2184,10 @@
         <v>106</v>
       </c>
       <c r="I31" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="J31">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="K31">
         <v>106</v>
@@ -2200,7 +2202,7 @@
         <v>19</v>
       </c>
       <c r="O31" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
@@ -2229,10 +2231,10 @@
         <v>140</v>
       </c>
       <c r="I32" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J32">
-        <v>132</v>
+        <v>103</v>
       </c>
       <c r="K32">
         <v>140</v>
@@ -2247,7 +2249,7 @@
         <v>19</v>
       </c>
       <c r="O32" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
@@ -2276,10 +2278,10 @@
         <v>140</v>
       </c>
       <c r="I33" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="J33">
-        <v>131</v>
+        <v>99</v>
       </c>
       <c r="K33">
         <v>140</v>
@@ -2291,10 +2293,10 @@
         <v>11</v>
       </c>
       <c r="N33" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="O33" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
@@ -2323,10 +2325,10 @@
         <v>125</v>
       </c>
       <c r="I34" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="J34">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="K34">
         <v>125</v>
@@ -2341,7 +2343,7 @@
         <v>19</v>
       </c>
       <c r="O34" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
@@ -2370,10 +2372,10 @@
         <v>94</v>
       </c>
       <c r="I35" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J35">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="K35">
         <v>94</v>
@@ -2385,10 +2387,10 @@
         <v>12</v>
       </c>
       <c r="N35" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="O35" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
@@ -2417,10 +2419,10 @@
         <v>101</v>
       </c>
       <c r="I36" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J36">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K36">
         <v>101</v>
@@ -2432,10 +2434,10 @@
         <v>6</v>
       </c>
       <c r="N36" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="O36" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
@@ -2464,10 +2466,10 @@
         <v>144</v>
       </c>
       <c r="I37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="J37">
-        <v>129</v>
+        <v>70</v>
       </c>
       <c r="K37">
         <v>144</v>
@@ -2479,10 +2481,10 @@
         <v>10</v>
       </c>
       <c r="N37" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="O37" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
@@ -2511,10 +2513,10 @@
         <v>121</v>
       </c>
       <c r="I38" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J38">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="K38">
         <v>121</v>
@@ -2526,10 +2528,10 @@
         <v>4</v>
       </c>
       <c r="N38" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="O38" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
@@ -2558,10 +2560,10 @@
         <v>126</v>
       </c>
       <c r="I39" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="J39">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="K39">
         <v>126</v>
@@ -2576,7 +2578,7 @@
         <v>19</v>
       </c>
       <c r="O39" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
@@ -2605,10 +2607,10 @@
         <v>110</v>
       </c>
       <c r="I40" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="J40">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="K40">
         <v>110</v>
@@ -2623,7 +2625,7 @@
         <v>19</v>
       </c>
       <c r="O40" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
@@ -2652,10 +2654,10 @@
         <v>87</v>
       </c>
       <c r="I41" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="J41">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="K41">
         <v>87</v>
@@ -2670,7 +2672,7 @@
         <v>19</v>
       </c>
       <c r="O41" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
@@ -2699,10 +2701,10 @@
         <v>103</v>
       </c>
       <c r="I42" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J42">
-        <v>81</v>
+        <v>41</v>
       </c>
       <c r="K42">
         <v>103</v>
@@ -2717,7 +2719,7 @@
         <v>19</v>
       </c>
       <c r="O42" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2726,6 +2728,2079 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B917C4BF-6827-4C36-8E4A-9DB98CA460B6}">
+  <dimension ref="A1:O23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>42372845</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>19</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>7</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>37</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2">
+        <v>14</v>
+      </c>
+      <c r="K2">
+        <v>37</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>8</v>
+      </c>
+      <c r="N2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>42381392</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>86</v>
+      </c>
+      <c r="D3">
+        <v>21</v>
+      </c>
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>115</v>
+      </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3">
+        <v>58</v>
+      </c>
+      <c r="K3">
+        <v>115</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>11</v>
+      </c>
+      <c r="N3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>42406507</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>184</v>
+      </c>
+      <c r="D4">
+        <v>46</v>
+      </c>
+      <c r="E4">
+        <v>27</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
+      </c>
+      <c r="H4">
+        <v>262</v>
+      </c>
+      <c r="I4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4">
+        <v>66</v>
+      </c>
+      <c r="K4">
+        <v>262</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>38</v>
+      </c>
+      <c r="N4" t="s">
+        <v>19</v>
+      </c>
+      <c r="O4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>42426592</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>128</v>
+      </c>
+      <c r="D5">
+        <v>54</v>
+      </c>
+      <c r="E5">
+        <v>19</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>204</v>
+      </c>
+      <c r="I5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5">
+        <v>70</v>
+      </c>
+      <c r="K5">
+        <v>204</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>55</v>
+      </c>
+      <c r="N5" t="s">
+        <v>19</v>
+      </c>
+      <c r="O5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>42426641</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>178</v>
+      </c>
+      <c r="D6">
+        <v>25</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>215</v>
+      </c>
+      <c r="I6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J6">
+        <v>125</v>
+      </c>
+      <c r="K6">
+        <v>215</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>29</v>
+      </c>
+      <c r="N6" t="s">
+        <v>19</v>
+      </c>
+      <c r="O6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>42458992</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>22</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>26</v>
+      </c>
+      <c r="I7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7">
+        <v>17</v>
+      </c>
+      <c r="K7">
+        <v>26</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+      <c r="N7" t="s">
+        <v>19</v>
+      </c>
+      <c r="O7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>42459041</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>12</v>
+      </c>
+      <c r="D8">
+        <v>8</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>23</v>
+      </c>
+      <c r="I8" t="s">
+        <v>29</v>
+      </c>
+      <c r="J8">
+        <v>7</v>
+      </c>
+      <c r="K8">
+        <v>23</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>6</v>
+      </c>
+      <c r="N8" t="s">
+        <v>19</v>
+      </c>
+      <c r="O8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>42459099</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>47</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>49</v>
+      </c>
+      <c r="I9" t="s">
+        <v>31</v>
+      </c>
+      <c r="J9">
+        <v>19</v>
+      </c>
+      <c r="K9">
+        <v>49</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>4</v>
+      </c>
+      <c r="N9" t="s">
+        <v>19</v>
+      </c>
+      <c r="O9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>42459241</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>37</v>
+      </c>
+      <c r="D10">
+        <v>22</v>
+      </c>
+      <c r="E10">
+        <v>6</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>2</v>
+      </c>
+      <c r="H10">
+        <v>68</v>
+      </c>
+      <c r="I10" t="s">
+        <v>33</v>
+      </c>
+      <c r="J10">
+        <v>18</v>
+      </c>
+      <c r="K10">
+        <v>68</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>35</v>
+      </c>
+      <c r="N10" t="s">
+        <v>19</v>
+      </c>
+      <c r="O10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>42459298</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>20</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>26</v>
+      </c>
+      <c r="I11" t="s">
+        <v>35</v>
+      </c>
+      <c r="J11">
+        <v>15</v>
+      </c>
+      <c r="K11">
+        <v>26</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>2</v>
+      </c>
+      <c r="N11" t="s">
+        <v>19</v>
+      </c>
+      <c r="O11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>42463024</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>301</v>
+      </c>
+      <c r="D12">
+        <v>31</v>
+      </c>
+      <c r="E12">
+        <v>11</v>
+      </c>
+      <c r="F12">
+        <v>4</v>
+      </c>
+      <c r="G12">
+        <v>5</v>
+      </c>
+      <c r="H12">
+        <v>353</v>
+      </c>
+      <c r="I12" t="s">
+        <v>37</v>
+      </c>
+      <c r="J12">
+        <v>103</v>
+      </c>
+      <c r="K12">
+        <v>353</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>53</v>
+      </c>
+      <c r="N12" t="s">
+        <v>19</v>
+      </c>
+      <c r="O12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>42463063</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>209</v>
+      </c>
+      <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>7</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13">
+        <v>228</v>
+      </c>
+      <c r="I13" t="s">
+        <v>39</v>
+      </c>
+      <c r="J13">
+        <v>100</v>
+      </c>
+      <c r="K13">
+        <v>228</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>108</v>
+      </c>
+      <c r="N13" t="s">
+        <v>19</v>
+      </c>
+      <c r="O13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>42705635</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>110</v>
+      </c>
+      <c r="D14">
+        <v>60</v>
+      </c>
+      <c r="E14">
+        <v>21</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>195</v>
+      </c>
+      <c r="I14" t="s">
+        <v>41</v>
+      </c>
+      <c r="J14">
+        <v>65</v>
+      </c>
+      <c r="K14">
+        <v>195</v>
+      </c>
+      <c r="L14">
+        <v>3</v>
+      </c>
+      <c r="M14">
+        <v>20</v>
+      </c>
+      <c r="N14" t="s">
+        <v>42</v>
+      </c>
+      <c r="O14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>42731028</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>167</v>
+      </c>
+      <c r="D15">
+        <v>20</v>
+      </c>
+      <c r="E15">
+        <v>12</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>201</v>
+      </c>
+      <c r="I15" t="s">
+        <v>44</v>
+      </c>
+      <c r="J15">
+        <v>99</v>
+      </c>
+      <c r="K15">
+        <v>201</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>15</v>
+      </c>
+      <c r="N15" t="s">
+        <v>45</v>
+      </c>
+      <c r="O15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>42913719</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>148</v>
+      </c>
+      <c r="D16">
+        <v>36</v>
+      </c>
+      <c r="E16">
+        <v>10</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>196</v>
+      </c>
+      <c r="I16" t="s">
+        <v>47</v>
+      </c>
+      <c r="J16">
+        <v>142</v>
+      </c>
+      <c r="K16">
+        <v>196</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>25</v>
+      </c>
+      <c r="N16" t="s">
+        <v>48</v>
+      </c>
+      <c r="O16" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>42971568</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <v>102</v>
+      </c>
+      <c r="D17">
+        <v>23</v>
+      </c>
+      <c r="E17">
+        <v>6</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>132</v>
+      </c>
+      <c r="I17" t="s">
+        <v>50</v>
+      </c>
+      <c r="J17">
+        <v>97</v>
+      </c>
+      <c r="K17">
+        <v>132</v>
+      </c>
+      <c r="L17">
+        <v>2</v>
+      </c>
+      <c r="M17">
+        <v>12</v>
+      </c>
+      <c r="N17" t="s">
+        <v>51</v>
+      </c>
+      <c r="O17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>42997602</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>148</v>
+      </c>
+      <c r="D18">
+        <v>33</v>
+      </c>
+      <c r="E18">
+        <v>13</v>
+      </c>
+      <c r="F18">
+        <v>2</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>197</v>
+      </c>
+      <c r="I18" t="s">
+        <v>53</v>
+      </c>
+      <c r="J18">
+        <v>97</v>
+      </c>
+      <c r="K18">
+        <v>197</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>17</v>
+      </c>
+      <c r="N18" t="s">
+        <v>48</v>
+      </c>
+      <c r="O18" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>43022614</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>114</v>
+      </c>
+      <c r="D19">
+        <v>31</v>
+      </c>
+      <c r="E19">
+        <v>18</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>165</v>
+      </c>
+      <c r="I19" t="s">
+        <v>55</v>
+      </c>
+      <c r="J19">
+        <v>109</v>
+      </c>
+      <c r="K19">
+        <v>165</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19">
+        <v>35</v>
+      </c>
+      <c r="N19" t="s">
+        <v>56</v>
+      </c>
+      <c r="O19" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>43081554</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>73</v>
+      </c>
+      <c r="D20">
+        <v>40</v>
+      </c>
+      <c r="E20">
+        <v>20</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>134</v>
+      </c>
+      <c r="I20" t="s">
+        <v>58</v>
+      </c>
+      <c r="J20">
+        <v>66</v>
+      </c>
+      <c r="K20">
+        <v>134</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20">
+        <v>24</v>
+      </c>
+      <c r="N20" t="s">
+        <v>59</v>
+      </c>
+      <c r="O20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>43110506</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>86</v>
+      </c>
+      <c r="D21">
+        <v>22</v>
+      </c>
+      <c r="E21">
+        <v>8</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>119</v>
+      </c>
+      <c r="I21" t="s">
+        <v>61</v>
+      </c>
+      <c r="J21">
+        <v>81</v>
+      </c>
+      <c r="K21">
+        <v>119</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21">
+        <v>18</v>
+      </c>
+      <c r="N21" t="s">
+        <v>62</v>
+      </c>
+      <c r="O21" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>43138108</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>102</v>
+      </c>
+      <c r="D22">
+        <v>38</v>
+      </c>
+      <c r="E22">
+        <v>12</v>
+      </c>
+      <c r="F22">
+        <v>2</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>155</v>
+      </c>
+      <c r="I22" t="s">
+        <v>64</v>
+      </c>
+      <c r="J22">
+        <v>76</v>
+      </c>
+      <c r="K22">
+        <v>155</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22">
+        <v>25</v>
+      </c>
+      <c r="N22" t="s">
+        <v>19</v>
+      </c>
+      <c r="O22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>43166702</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>107</v>
+      </c>
+      <c r="D23">
+        <v>47</v>
+      </c>
+      <c r="E23">
+        <v>11</v>
+      </c>
+      <c r="F23">
+        <v>2</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>168</v>
+      </c>
+      <c r="I23" t="s">
+        <v>66</v>
+      </c>
+      <c r="J23">
+        <v>81</v>
+      </c>
+      <c r="K23">
+        <v>168</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+      <c r="M23">
+        <v>15</v>
+      </c>
+      <c r="N23" t="s">
+        <v>67</v>
+      </c>
+      <c r="O23" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D93C4E66-FBE9-4925-8D98-3112F0EA52DB}">
+  <dimension ref="A1:O20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>8200826</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>134</v>
+      </c>
+      <c r="D2">
+        <v>27</v>
+      </c>
+      <c r="E2">
+        <v>33</v>
+      </c>
+      <c r="F2">
+        <v>28</v>
+      </c>
+      <c r="G2">
+        <v>36</v>
+      </c>
+      <c r="H2">
+        <v>259</v>
+      </c>
+      <c r="I2" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2">
+        <v>6</v>
+      </c>
+      <c r="K2">
+        <v>4116</v>
+      </c>
+      <c r="L2">
+        <v>816</v>
+      </c>
+      <c r="M2">
+        <v>2050</v>
+      </c>
+      <c r="N2" t="s">
+        <v>117</v>
+      </c>
+      <c r="O2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>43230061</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>91</v>
+      </c>
+      <c r="D3">
+        <v>33</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>130</v>
+      </c>
+      <c r="I3" t="s">
+        <v>70</v>
+      </c>
+      <c r="J3">
+        <v>77</v>
+      </c>
+      <c r="K3">
+        <v>130</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>54</v>
+      </c>
+      <c r="N3" t="s">
+        <v>19</v>
+      </c>
+      <c r="O3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>43290314</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>88</v>
+      </c>
+      <c r="D4">
+        <v>34</v>
+      </c>
+      <c r="E4">
+        <v>9</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>133</v>
+      </c>
+      <c r="I4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J4">
+        <v>72</v>
+      </c>
+      <c r="K4">
+        <v>133</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>30</v>
+      </c>
+      <c r="N4" t="s">
+        <v>59</v>
+      </c>
+      <c r="O4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>43319297</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>63</v>
+      </c>
+      <c r="D5">
+        <v>26</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>101</v>
+      </c>
+      <c r="I5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J5">
+        <v>50</v>
+      </c>
+      <c r="K5">
+        <v>101</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>6</v>
+      </c>
+      <c r="N5" t="s">
+        <v>19</v>
+      </c>
+      <c r="O5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>43346700</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>101</v>
+      </c>
+      <c r="D6">
+        <v>16</v>
+      </c>
+      <c r="E6">
+        <v>7</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>126</v>
+      </c>
+      <c r="I6" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6">
+        <v>77</v>
+      </c>
+      <c r="K6">
+        <v>126</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>16</v>
+      </c>
+      <c r="N6" t="s">
+        <v>19</v>
+      </c>
+      <c r="O6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>43374604</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>61</v>
+      </c>
+      <c r="D7">
+        <v>15</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>80</v>
+      </c>
+      <c r="I7" t="s">
+        <v>78</v>
+      </c>
+      <c r="J7">
+        <v>56</v>
+      </c>
+      <c r="K7">
+        <v>80</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>8</v>
+      </c>
+      <c r="N7" t="s">
+        <v>19</v>
+      </c>
+      <c r="O7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>43402439</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>96</v>
+      </c>
+      <c r="D8">
+        <v>26</v>
+      </c>
+      <c r="E8">
+        <v>6</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>130</v>
+      </c>
+      <c r="I8" t="s">
+        <v>80</v>
+      </c>
+      <c r="J8">
+        <v>89</v>
+      </c>
+      <c r="K8">
+        <v>130</v>
+      </c>
+      <c r="L8">
+        <v>5</v>
+      </c>
+      <c r="M8">
+        <v>4</v>
+      </c>
+      <c r="N8" t="s">
+        <v>28</v>
+      </c>
+      <c r="O8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>43430885</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>75</v>
+      </c>
+      <c r="D9">
+        <v>22</v>
+      </c>
+      <c r="E9">
+        <v>7</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>106</v>
+      </c>
+      <c r="I9" t="s">
+        <v>82</v>
+      </c>
+      <c r="J9">
+        <v>70</v>
+      </c>
+      <c r="K9">
+        <v>106</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>6</v>
+      </c>
+      <c r="N9" t="s">
+        <v>19</v>
+      </c>
+      <c r="O9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>43539274</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>110</v>
+      </c>
+      <c r="D10">
+        <v>24</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>140</v>
+      </c>
+      <c r="I10" t="s">
+        <v>84</v>
+      </c>
+      <c r="J10">
+        <v>103</v>
+      </c>
+      <c r="K10">
+        <v>140</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>11</v>
+      </c>
+      <c r="N10" t="s">
+        <v>19</v>
+      </c>
+      <c r="O10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>43566043</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>107</v>
+      </c>
+      <c r="D11">
+        <v>28</v>
+      </c>
+      <c r="E11">
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>140</v>
+      </c>
+      <c r="I11" t="s">
+        <v>86</v>
+      </c>
+      <c r="J11">
+        <v>99</v>
+      </c>
+      <c r="K11">
+        <v>140</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>11</v>
+      </c>
+      <c r="N11" t="s">
+        <v>87</v>
+      </c>
+      <c r="O11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>43593087</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>97</v>
+      </c>
+      <c r="D12">
+        <v>26</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>125</v>
+      </c>
+      <c r="I12" t="s">
+        <v>88</v>
+      </c>
+      <c r="J12">
+        <v>92</v>
+      </c>
+      <c r="K12">
+        <v>125</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>8</v>
+      </c>
+      <c r="N12" t="s">
+        <v>19</v>
+      </c>
+      <c r="O12" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>43614456</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>68</v>
+      </c>
+      <c r="D13">
+        <v>20</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>94</v>
+      </c>
+      <c r="I13" t="s">
+        <v>90</v>
+      </c>
+      <c r="J13">
+        <v>61</v>
+      </c>
+      <c r="K13">
+        <v>94</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13">
+        <v>12</v>
+      </c>
+      <c r="N13" t="s">
+        <v>91</v>
+      </c>
+      <c r="O13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>43674483</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>84</v>
+      </c>
+      <c r="D14">
+        <v>13</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>101</v>
+      </c>
+      <c r="I14" t="s">
+        <v>93</v>
+      </c>
+      <c r="J14">
+        <v>79</v>
+      </c>
+      <c r="K14">
+        <v>101</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>6</v>
+      </c>
+      <c r="N14" t="s">
+        <v>94</v>
+      </c>
+      <c r="O14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>43862968</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>117</v>
+      </c>
+      <c r="D15">
+        <v>23</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>144</v>
+      </c>
+      <c r="I15" t="s">
+        <v>95</v>
+      </c>
+      <c r="J15">
+        <v>70</v>
+      </c>
+      <c r="K15">
+        <v>144</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>10</v>
+      </c>
+      <c r="N15" t="s">
+        <v>96</v>
+      </c>
+      <c r="O15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>43891958</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>87</v>
+      </c>
+      <c r="D16">
+        <v>30</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>121</v>
+      </c>
+      <c r="I16" t="s">
+        <v>98</v>
+      </c>
+      <c r="J16">
+        <v>82</v>
+      </c>
+      <c r="K16">
+        <v>121</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>4</v>
+      </c>
+      <c r="N16" t="s">
+        <v>99</v>
+      </c>
+      <c r="O16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>43920615</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17">
+        <v>96</v>
+      </c>
+      <c r="D17">
+        <v>27</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>126</v>
+      </c>
+      <c r="I17" t="s">
+        <v>101</v>
+      </c>
+      <c r="J17">
+        <v>91</v>
+      </c>
+      <c r="K17">
+        <v>126</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>8</v>
+      </c>
+      <c r="N17" t="s">
+        <v>19</v>
+      </c>
+      <c r="O17" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>43949404</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18">
+        <v>79</v>
+      </c>
+      <c r="D18">
+        <v>26</v>
+      </c>
+      <c r="E18">
+        <v>3</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>110</v>
+      </c>
+      <c r="I18" t="s">
+        <v>103</v>
+      </c>
+      <c r="J18">
+        <v>74</v>
+      </c>
+      <c r="K18">
+        <v>110</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>5</v>
+      </c>
+      <c r="N18" t="s">
+        <v>19</v>
+      </c>
+      <c r="O18" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>43978801</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>65</v>
+      </c>
+      <c r="D19">
+        <v>19</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>87</v>
+      </c>
+      <c r="I19" t="s">
+        <v>105</v>
+      </c>
+      <c r="J19">
+        <v>60</v>
+      </c>
+      <c r="K19">
+        <v>87</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>12</v>
+      </c>
+      <c r="N19" t="s">
+        <v>19</v>
+      </c>
+      <c r="O19" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>44010401</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20">
+        <v>62</v>
+      </c>
+      <c r="D20">
+        <v>36</v>
+      </c>
+      <c r="E20">
+        <v>2</v>
+      </c>
+      <c r="F20">
+        <v>2</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>103</v>
+      </c>
+      <c r="I20" t="s">
+        <v>107</v>
+      </c>
+      <c r="J20">
+        <v>41</v>
+      </c>
+      <c r="K20">
+        <v>103</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>5</v>
+      </c>
+      <c r="N20" t="s">
+        <v>19</v>
+      </c>
+      <c r="O20" t="s">
+        <v>108</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4719527-41BF-4F40-B12E-62783B3C5FD2}">
   <dimension ref="A1:G52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2741,13 +4816,13 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -2755,10 +4830,10 @@
         <v>36425882</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -2766,10 +4841,10 @@
         <v>2542992</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -2777,19 +4852,19 @@
         <v>3158809</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>118</v>
-      </c>
       <c r="F4" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -2797,10 +4872,10 @@
         <v>3281810</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E5" s="1">
         <f>COUNTA(C2:C52)</f>
@@ -2820,10 +4895,10 @@
         <v>3415189</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F6" s="2">
         <f>F5/E5</f>
@@ -2839,10 +4914,10 @@
         <v>3434386</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -2850,10 +4925,10 @@
         <v>3531594</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
@@ -2861,10 +4936,10 @@
         <v>3819032</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -2872,10 +4947,10 @@
         <v>4167618</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -2883,10 +4958,10 @@
         <v>4179701</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -2894,10 +4969,10 @@
         <v>4188518</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -2905,10 +4980,10 @@
         <v>4253659</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -2916,10 +4991,10 @@
         <v>4276951</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -2927,10 +5002,10 @@
         <v>4726514</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -2938,10 +5013,10 @@
         <v>42011766</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -2949,10 +5024,10 @@
         <v>42011817</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -2960,10 +5035,10 @@
         <v>42012426</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -2971,10 +5046,10 @@
         <v>42077631</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -2982,10 +5057,10 @@
         <v>42426592</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -2993,10 +5068,10 @@
         <v>42426641</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -3004,10 +5079,10 @@
         <v>42758642</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -3015,10 +5090,10 @@
         <v>42787717</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -3026,10 +5101,10 @@
         <v>42406507</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -3037,10 +5112,10 @@
         <v>42598944</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -3048,10 +5123,10 @@
         <v>42459099</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -3059,10 +5134,10 @@
         <v>42459206</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -3070,10 +5145,10 @@
         <v>42459241</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -3081,10 +5156,10 @@
         <v>42459298</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -3092,10 +5167,10 @@
         <v>42458992</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -3103,10 +5178,10 @@
         <v>42459148</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -3114,10 +5189,10 @@
         <v>42705635</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -3125,10 +5200,10 @@
         <v>43022302</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -3136,10 +5211,10 @@
         <v>43022440</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -3147,10 +5222,10 @@
         <v>43375656</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -3158,10 +5233,10 @@
         <v>16372934</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -3169,10 +5244,10 @@
         <v>3463245</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -3180,10 +5255,10 @@
         <v>3711577</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -3191,10 +5266,10 @@
         <v>3728922</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -3202,10 +5277,10 @@
         <v>3754003</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -3213,10 +5288,10 @@
         <v>4239307</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -3224,10 +5299,10 @@
         <v>31956677</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -3235,10 +5310,10 @@
         <v>42010347</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -3246,10 +5321,10 @@
         <v>42012522</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -3257,10 +5332,10 @@
         <v>42079879</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -3268,10 +5343,10 @@
         <v>42814075</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -3279,10 +5354,10 @@
         <v>43110281</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
@@ -3290,10 +5365,10 @@
         <v>42459041</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -3301,10 +5376,10 @@
         <v>42463063</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
@@ -3312,10 +5387,10 @@
         <v>42463024</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -3323,10 +5398,10 @@
         <v>42731028</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -3334,10 +5409,10 @@
         <v>43613297</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update latest simulation analysis (resimulate to fit Avira strat observation criteria)
</commit_message>
<xml_diff>
--- a/data/Simulation_User_Summary.xlsx
+++ b/data/Simulation_User_Summary.xlsx
@@ -8,18 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wei.kc\Desktop\Adhoc\03 Sept 2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD14C98E-C8D4-4114-A213-EF76DD6EC84D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C210539-21B2-48E6-B69B-4D9A7A77D6FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="737" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="user-summary (July_Aug2026)" sheetId="1" r:id="rId1"/>
-    <sheet name="user-summary(July2026)" sheetId="3" r:id="rId2"/>
-    <sheet name="user-summary(Aug2026)" sheetId="4" r:id="rId3"/>
-    <sheet name="linkage" sheetId="2" r:id="rId4"/>
+    <sheet name="account_info" sheetId="5" r:id="rId2"/>
+    <sheet name="user-summary(July2026)" sheetId="3" r:id="rId3"/>
+    <sheet name="user-summary(Aug2026)" sheetId="4" r:id="rId4"/>
+    <sheet name="linkage" sheetId="2" r:id="rId5"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
+  </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">linkage!$A$1:$C$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">account_info!$A$1:$G$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">linkage!$A$1:$H$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'user-summary (July_Aug2026)'!$A$1:$O$42</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="134">
   <si>
     <t>user_id</t>
   </si>
@@ -399,13 +406,61 @@
   </si>
   <si>
     <t>49.81%</t>
+  </si>
+  <si>
+    <t>register_time</t>
+  </si>
+  <si>
+    <t>ban_status</t>
+  </si>
+  <si>
+    <t>NOT BAN</t>
+  </si>
+  <si>
+    <t>BANNED</t>
+  </si>
+  <si>
+    <t>ban_reason</t>
+  </si>
+  <si>
+    <t>ban_datetime</t>
+  </si>
+  <si>
+    <t>FTU đặt hơn 23 đơn hàng, địa chỉ không cụ thể, các TX đều không liên hệ được</t>
+  </si>
+  <si>
+    <t>FTU đặt hơn 60 đơn hàng, địa chỉ không cụ thể, các TX đều không liên hệ được</t>
+  </si>
+  <si>
+    <t>3538384917878756304 đơn phá</t>
+  </si>
+  <si>
+    <t>3539101478889410627 - FAKE ORDER</t>
+  </si>
+  <si>
+    <t>is_corp</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Corp</t>
+  </si>
+  <si>
+    <t>lifetime_completion_rate</t>
+  </si>
+  <si>
+    <t>target_user_id</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -420,6 +475,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -429,7 +498,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -437,20 +506,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDEE0E3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDEE0E3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDEE0E3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDEE0E3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="22" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{C269E39C-30EE-4724-A890-6E0172D544BA}"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Percent 2" xfId="2" xr:uid="{370C1C47-7B54-4911-9F66-BE60333CAA84}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -464,6 +557,721 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Results export"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="2">
+          <cell r="C2" t="str">
+            <v>2026-08-06 10:06:49</v>
+          </cell>
+          <cell r="F2" t="str">
+            <v>43374604</v>
+          </cell>
+          <cell r="G2" t="str">
+            <v>FTU đặt hơn 40 đơn phá</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="C3" t="str">
+            <v>2026-08-25 09:35:57</v>
+          </cell>
+          <cell r="F3" t="str">
+            <v>43891958</v>
+          </cell>
+          <cell r="G3" t="str">
+            <v>disruptive user, more than 20 fake orders</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="C4" t="str">
+            <v>2026-08-24 10:23:29</v>
+          </cell>
+          <cell r="F4" t="str">
+            <v>43862968</v>
+          </cell>
+          <cell r="G4" t="str">
+            <v>disruptive user, more than 20 fake orders</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="C5" t="str">
+            <v>2026-07-22 10:24:05</v>
+          </cell>
+          <cell r="F5" t="str">
+            <v>42459099</v>
+          </cell>
+          <cell r="G5" t="str">
+            <v>Fake order - Đặt 49 đơn liên tục, địa chỉ ko chính xác, tài xế không liên hệ được</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="C6" t="str">
+            <v>2026-07-22 12:09:47</v>
+          </cell>
+          <cell r="F6" t="str">
+            <v>42426641</v>
+          </cell>
+          <cell r="G6" t="str">
+            <v>Fake orders - FTU đặt hơn 200 đơn hàng, địa chỉ không cụ thể, các TX đều không liên hệ được</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="C7" t="str">
+            <v>2026-07-22 12:10:28</v>
+          </cell>
+          <cell r="F7" t="str">
+            <v>42406507</v>
+          </cell>
+          <cell r="G7" t="str">
+            <v>Fake orders - FTU đặt hơn 200 đơn hàng, địa chỉ không cụ thể, các TX đều không liên hệ được</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="C8" t="str">
+            <v>2026-07-23 11:30:19</v>
+          </cell>
+          <cell r="F8" t="str">
+            <v>42971568</v>
+          </cell>
+          <cell r="G8" t="str">
+            <v>FTU đặt hơn 100 đơn phá, các TX đến nơi không liên hệ được</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="C9" t="str">
+            <v>2026-07-24 10:24:04</v>
+          </cell>
+          <cell r="F9" t="str">
+            <v>42997602</v>
+          </cell>
+          <cell r="G9" t="str">
+            <v>FTU đặt hơn 200 đơn hàng, địa chỉ không cụ thể, các TX đều không liên hệ được</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="C10" t="str">
+            <v>2026-08-15 10:07:41</v>
+          </cell>
+          <cell r="F10" t="str">
+            <v>43614456</v>
+          </cell>
+          <cell r="G10" t="str">
+            <v>FTU placed over 100 disruptive order</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="C11" t="str">
+            <v>2026-08-17 08:56:06</v>
+          </cell>
+          <cell r="F11" t="str">
+            <v>43674483</v>
+          </cell>
+          <cell r="G11" t="str">
+            <v>disruptive user, more than 20 fake orders</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="C12" t="str">
+            <v>2026-08-10 10:29:23</v>
+          </cell>
+          <cell r="F12" t="str">
+            <v>43430885</v>
+          </cell>
+          <cell r="G12" t="str">
+            <v>FTU placed over 100 disruptive orders</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="C13" t="str">
+            <v>2026-08-01 10:01:46</v>
+          </cell>
+          <cell r="F13" t="str">
+            <v>43230061</v>
+          </cell>
+          <cell r="G13" t="str">
+            <v>FTU đặt hơn 100 đơn phá</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="C14" t="str">
+            <v>2026-08-04 10:10:58</v>
+          </cell>
+          <cell r="F14" t="str">
+            <v>43319297</v>
+          </cell>
+          <cell r="G14" t="str">
+            <v>FTU đặt hơn 100 đơn phá</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="C15" t="str">
+            <v>2026-07-30 10:00:09</v>
+          </cell>
+          <cell r="F15" t="str">
+            <v>43166702</v>
+          </cell>
+          <cell r="G15" t="str">
+            <v>Disruptive user, TX Phạm Minh Truyền 2852976 báo cáo Kh 43166702 đặt phá</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="C16" t="str">
+            <v>2026-07-27 10:39:43</v>
+          </cell>
+          <cell r="F16" t="str">
+            <v>43022614</v>
+          </cell>
+          <cell r="G16" t="str">
+            <v>User đặt hơn 160 đơn phá, các TX đều không liên hệ được</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="C17" t="str">
+            <v>2026-08-28 10:10:00</v>
+          </cell>
+          <cell r="F17" t="str">
+            <v>43978801</v>
+          </cell>
+          <cell r="G17" t="str">
+            <v>Placed more than 80 fake orders</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="C18" t="str">
+            <v>2026-08-03 10:24:03</v>
+          </cell>
+          <cell r="F18" t="str">
+            <v>43290314</v>
+          </cell>
+          <cell r="G18" t="str">
+            <v>FTU đặt hơn 100 đơn phá. Offensive user's name</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="C19" t="str">
+            <v>2026-07-22 10:10:28</v>
+          </cell>
+          <cell r="F19" t="str">
+            <v>42463024</v>
+          </cell>
+          <cell r="G19" t="str">
+            <v>Fake orders. Đặt 61 đơn trong 3 ngày, không liên hệ được</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="C20" t="str">
+            <v>2026-07-22 10:25:04</v>
+          </cell>
+          <cell r="F20" t="str">
+            <v>42913719</v>
+          </cell>
+          <cell r="G20" t="str">
+            <v>Fake order - Corp đặt 200 đơn phá, các TX đều ko liên hệ được</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="C21" t="str">
+            <v>2026-08-12 10:27:38</v>
+          </cell>
+          <cell r="F21" t="str">
+            <v>43539274</v>
+          </cell>
+          <cell r="G21" t="str">
+            <v>FTU placed over 100 disruptive order</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="C22" t="str">
+            <v>2026-07-29 09:27:17</v>
+          </cell>
+          <cell r="F22" t="str">
+            <v>43138108</v>
+          </cell>
+          <cell r="G22" t="str">
+            <v>disruptive user, TX Phạm Minh Truyền 2852976 báo cáo Kh 43138108 đặt phá đơn</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="C23" t="str">
+            <v>2026-08-26 10:16:44</v>
+          </cell>
+          <cell r="F23" t="str">
+            <v>43920615</v>
+          </cell>
+          <cell r="G23" t="str">
+            <v>Placed more than 100 fake orders</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="C24" t="str">
+            <v>2026-08-05 10:13:34</v>
+          </cell>
+          <cell r="F24" t="str">
+            <v>43346700</v>
+          </cell>
+          <cell r="G24" t="str">
+            <v>User đặt hơn 100 đơn phá</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="C25" t="str">
+            <v>2026-08-27 11:18:17</v>
+          </cell>
+          <cell r="F25" t="str">
+            <v>43949404</v>
+          </cell>
+          <cell r="G25" t="str">
+            <v>Placed over 100 fake orders</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="C26" t="str">
+            <v>2026-08-13 10:16:23</v>
+          </cell>
+          <cell r="F26" t="str">
+            <v>43566043</v>
+          </cell>
+          <cell r="G26" t="str">
+            <v>FTU placed over 100 disruptive order</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="C27" t="str">
+            <v>2026-07-28 09:56:11</v>
+          </cell>
+          <cell r="F27" t="str">
+            <v>43110506</v>
+          </cell>
+          <cell r="G27" t="str">
+            <v>disruptive user</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="C28" t="str">
+            <v>2026-08-07 10:35:45</v>
+          </cell>
+          <cell r="F28" t="str">
+            <v>43402439</v>
+          </cell>
+          <cell r="G28" t="str">
+            <v>FTU placed over 100 disruptive orders</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="C29" t="str">
+            <v>2026-08-31 10:06:07</v>
+          </cell>
+          <cell r="F29" t="str">
+            <v>44010401</v>
+          </cell>
+          <cell r="G29" t="str">
+            <v>Placed over 100 fake orders</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="C30" t="str">
+            <v>2026-07-27 09:06:11</v>
+          </cell>
+          <cell r="F30" t="str">
+            <v>43081554</v>
+          </cell>
+          <cell r="G30" t="str">
+            <v>disruptive user, more than 20 fake orders</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="C31" t="str">
+            <v>2026-07-07 16:34:11</v>
+          </cell>
+          <cell r="F31" t="str">
+            <v>42463063</v>
+          </cell>
+          <cell r="G31" t="str">
+            <v>Disruptive user, banning and tagging under Platform Ops and MD approve</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="C32" t="str">
+            <v>2026-07-22 11:54:58</v>
+          </cell>
+          <cell r="F32" t="str">
+            <v>42426592</v>
+          </cell>
+          <cell r="G32" t="str">
+            <v>Fake order - FTU đặt hơn 200 đơn hàng, địa chỉ không cụ thể, các TX đều không liên hệ được</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="C33" t="str">
+            <v>2026-08-14 09:43:19</v>
+          </cell>
+          <cell r="F33" t="str">
+            <v>43593087</v>
+          </cell>
+          <cell r="G33" t="str">
+            <v>disruptive user</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Results export"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="2">
+          <cell r="A2">
+            <v>43319297</v>
+          </cell>
+          <cell r="R2">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="A3">
+            <v>42459099</v>
+          </cell>
+          <cell r="R3">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="A4">
+            <v>42459041</v>
+          </cell>
+          <cell r="R4">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="A5">
+            <v>42463024</v>
+          </cell>
+          <cell r="R5">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="A6">
+            <v>43674483</v>
+          </cell>
+          <cell r="R6">
+            <v>9.9009900990099011E-3</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="A7">
+            <v>42705635</v>
+          </cell>
+          <cell r="R7">
+            <v>1.5384615384615385E-2</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="A8">
+            <v>43138108</v>
+          </cell>
+          <cell r="R8">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="A9">
+            <v>43593087</v>
+          </cell>
+          <cell r="R9">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="A10">
+            <v>43862968</v>
+          </cell>
+          <cell r="R10">
+            <v>6.9444444444444441E-3</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="A11">
+            <v>43891958</v>
+          </cell>
+          <cell r="R11">
+            <v>8.2644628099173556E-3</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="A12">
+            <v>43290314</v>
+          </cell>
+          <cell r="R12">
+            <v>7.5187969924812026E-3</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="A13">
+            <v>42458992</v>
+          </cell>
+          <cell r="R13">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="A14">
+            <v>43110506</v>
+          </cell>
+          <cell r="R14">
+            <v>8.4033613445378148E-3</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="A15">
+            <v>44010401</v>
+          </cell>
+          <cell r="R15">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="A16">
+            <v>43346700</v>
+          </cell>
+          <cell r="R16">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="A17">
+            <v>42731028</v>
+          </cell>
+          <cell r="R17">
+            <v>4.9751243781094526E-3</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="A18">
+            <v>43978801</v>
+          </cell>
+          <cell r="R18">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="A19">
+            <v>42426592</v>
+          </cell>
+          <cell r="R19">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="A20">
+            <v>43166702</v>
+          </cell>
+          <cell r="R20">
+            <v>5.9523809523809521E-3</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="A21">
+            <v>43430885</v>
+          </cell>
+          <cell r="R21">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="A22">
+            <v>42426641</v>
+          </cell>
+          <cell r="R22">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="A23">
+            <v>42997602</v>
+          </cell>
+          <cell r="R23">
+            <v>5.076142131979695E-3</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="A24">
+            <v>43539274</v>
+          </cell>
+          <cell r="R24">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="A25">
+            <v>43566043</v>
+          </cell>
+          <cell r="R25">
+            <v>7.1428571428571426E-3</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="A26">
+            <v>42463063</v>
+          </cell>
+          <cell r="R26">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="A27">
+            <v>43022614</v>
+          </cell>
+          <cell r="R27">
+            <v>6.0606060606060606E-3</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="A28">
+            <v>42971568</v>
+          </cell>
+          <cell r="R28">
+            <v>1.5151515151515152E-2</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="A29">
+            <v>43081554</v>
+          </cell>
+          <cell r="R29">
+            <v>7.462686567164179E-3</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="A30">
+            <v>42459298</v>
+          </cell>
+          <cell r="R30">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="A31">
+            <v>43230061</v>
+          </cell>
+          <cell r="R31">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="A32">
+            <v>43920615</v>
+          </cell>
+          <cell r="R32">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="A33">
+            <v>42406507</v>
+          </cell>
+          <cell r="R33">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="34">
+          <cell r="A34">
+            <v>42913719</v>
+          </cell>
+          <cell r="R34">
+            <v>5.1020408163265302E-3</v>
+          </cell>
+        </row>
+        <row r="35">
+          <cell r="A35">
+            <v>42372845</v>
+          </cell>
+          <cell r="R35">
+            <v>2.7027027027027029E-2</v>
+          </cell>
+        </row>
+        <row r="36">
+          <cell r="A36">
+            <v>43949404</v>
+          </cell>
+          <cell r="R36">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="37">
+          <cell r="A37">
+            <v>43374604</v>
+          </cell>
+          <cell r="R37">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="38">
+          <cell r="A38">
+            <v>43402439</v>
+          </cell>
+          <cell r="R38">
+            <v>3.8461538461538464E-2</v>
+          </cell>
+        </row>
+        <row r="39">
+          <cell r="A39">
+            <v>43614456</v>
+          </cell>
+          <cell r="R39">
+            <v>1.0638297872340425E-2</v>
+          </cell>
+        </row>
+        <row r="40">
+          <cell r="A40">
+            <v>42459241</v>
+          </cell>
+          <cell r="R40">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="41">
+          <cell r="A41">
+            <v>42381392</v>
+          </cell>
+          <cell r="R41">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="42">
+          <cell r="A42">
+            <v>8200826</v>
+          </cell>
+          <cell r="R42">
+            <v>0.19748610103940054</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2723,11 +3531,1112 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O42" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB011E51-5698-4F7F-B1C8-99B7D0DBCADD}">
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="52.77734375" customWidth="1"/>
+    <col min="5" max="5" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>42372845</v>
+      </c>
+      <c r="B2" s="5">
+        <v>46203.812013888892</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" t="str">
+        <f>IF(C2="NOT BAN","",_xlfn.XLOOKUP(A2,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v/>
+      </c>
+      <c r="E2" s="6" t="str">
+        <f>IF(C2="NOT BAN","",_xlfn.XLOOKUP(A2,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v/>
+      </c>
+      <c r="F2" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="7">
+        <f>_xlfn.XLOOKUP(A2,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>2.7027027027027029E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>42381392</v>
+      </c>
+      <c r="B3" s="5">
+        <v>46204.304027777776</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" t="str">
+        <f>IF(C3="NOT BAN","",_xlfn.XLOOKUP(A3,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v/>
+      </c>
+      <c r="E3" s="6" t="str">
+        <f>IF(C3="NOT BAN","",_xlfn.XLOOKUP(A3,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v/>
+      </c>
+      <c r="F3" t="s">
+        <v>130</v>
+      </c>
+      <c r="G3" s="7">
+        <f>_xlfn.XLOOKUP(A3,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>42406507</v>
+      </c>
+      <c r="B4" s="5">
+        <v>46204.898495370369</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" t="e">
+        <f>IF(C4="NOT BAN","",_xlfn.XLOOKUP(A4,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E4" s="6" t="e">
+        <f>IF(C4="NOT BAN","",_xlfn.XLOOKUP(A4,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F4" t="s">
+        <v>130</v>
+      </c>
+      <c r="G4" s="7">
+        <f>_xlfn.XLOOKUP(A4,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>42426592</v>
+      </c>
+      <c r="B5" s="5">
+        <v>46205.677800925929</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" t="e">
+        <f>IF(C5="NOT BAN","",_xlfn.XLOOKUP(A5,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E5" s="6" t="e">
+        <f>IF(C5="NOT BAN","",_xlfn.XLOOKUP(A5,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F5" t="s">
+        <v>130</v>
+      </c>
+      <c r="G5" s="7">
+        <f>_xlfn.XLOOKUP(A5,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>42426641</v>
+      </c>
+      <c r="B6" s="5">
+        <v>46205.67900462963</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" t="e">
+        <f>IF(C6="NOT BAN","",_xlfn.XLOOKUP(A6,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E6" s="6" t="e">
+        <f>IF(C6="NOT BAN","",_xlfn.XLOOKUP(A6,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F6" t="s">
+        <v>130</v>
+      </c>
+      <c r="G6" s="7">
+        <f>_xlfn.XLOOKUP(A6,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>42458992</v>
+      </c>
+      <c r="B7" s="5">
+        <v>46206.779687499999</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" t="str">
+        <f>IF(C7="NOT BAN","",_xlfn.XLOOKUP(A7,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v/>
+      </c>
+      <c r="E7" s="6" t="str">
+        <f>IF(C7="NOT BAN","",_xlfn.XLOOKUP(A7,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v/>
+      </c>
+      <c r="F7" t="s">
+        <v>130</v>
+      </c>
+      <c r="G7" s="7">
+        <f>_xlfn.XLOOKUP(A7,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>42459041</v>
+      </c>
+      <c r="B8" s="5">
+        <v>46206.781064814815</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" t="s">
+        <v>125</v>
+      </c>
+      <c r="E8" s="6">
+        <v>46213.437199074076</v>
+      </c>
+      <c r="F8" t="s">
+        <v>130</v>
+      </c>
+      <c r="G8" s="7">
+        <f>_xlfn.XLOOKUP(A8,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>42459099</v>
+      </c>
+      <c r="B9" s="5">
+        <v>46206.782268518517</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" t="e">
+        <f>IF(C9="NOT BAN","",_xlfn.XLOOKUP(A9,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E9" s="6" t="e">
+        <f>IF(C9="NOT BAN","",_xlfn.XLOOKUP(A9,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F9" t="s">
+        <v>130</v>
+      </c>
+      <c r="G9" s="7">
+        <f>_xlfn.XLOOKUP(A9,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>42459241</v>
+      </c>
+      <c r="B10" s="5">
+        <v>46206.785729166666</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" t="s">
+        <v>126</v>
+      </c>
+      <c r="E10" s="6">
+        <v>46222.427881944444</v>
+      </c>
+      <c r="F10" t="s">
+        <v>130</v>
+      </c>
+      <c r="G10" s="7">
+        <f>_xlfn.XLOOKUP(A10,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>42459298</v>
+      </c>
+      <c r="B11" s="5">
+        <v>46206.787048611113</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" t="str">
+        <f>IF(C11="NOT BAN","",_xlfn.XLOOKUP(A11,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v/>
+      </c>
+      <c r="E11" s="6" t="str">
+        <f>IF(C11="NOT BAN","",_xlfn.XLOOKUP(A11,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v/>
+      </c>
+      <c r="F11" t="s">
+        <v>130</v>
+      </c>
+      <c r="G11" s="7">
+        <f>_xlfn.XLOOKUP(A11,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>42463024</v>
+      </c>
+      <c r="B12" s="5">
+        <v>46206.887523148151</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" t="e">
+        <f>IF(C12="NOT BAN","",_xlfn.XLOOKUP(A12,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E12" s="6" t="e">
+        <f>IF(C12="NOT BAN","",_xlfn.XLOOKUP(A12,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F12" t="s">
+        <v>131</v>
+      </c>
+      <c r="G12" s="7">
+        <f>_xlfn.XLOOKUP(A12,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
+        <v>42463063</v>
+      </c>
+      <c r="B13" s="5">
+        <v>46206.889074074075</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" t="e">
+        <f>IF(C13="NOT BAN","",_xlfn.XLOOKUP(A13,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E13" s="6" t="e">
+        <f>IF(C13="NOT BAN","",_xlfn.XLOOKUP(A13,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F13" t="s">
+        <v>131</v>
+      </c>
+      <c r="G13" s="7">
+        <f>_xlfn.XLOOKUP(A13,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
+        <v>42705635</v>
+      </c>
+      <c r="B14" s="5">
+        <v>46215.939513888887</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D14" t="s">
+        <v>127</v>
+      </c>
+      <c r="E14" s="6">
+        <v>46216.399270833332</v>
+      </c>
+      <c r="F14" t="s">
+        <v>130</v>
+      </c>
+      <c r="G14" s="7">
+        <f>_xlfn.XLOOKUP(A14,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>1.5384615384615385E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
+        <v>42731028</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46216.87908564815</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" t="s">
+        <v>128</v>
+      </c>
+      <c r="E15" s="6">
+        <v>46217.377581018518</v>
+      </c>
+      <c r="F15" t="s">
+        <v>130</v>
+      </c>
+      <c r="G15" s="7">
+        <f>_xlfn.XLOOKUP(A15,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>4.9751243781094526E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
+        <v>42913719</v>
+      </c>
+      <c r="B16" s="5">
+        <v>46223.899652777778</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D16" t="e">
+        <f>IF(C16="NOT BAN","",_xlfn.XLOOKUP(A16,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E16" s="6" t="e">
+        <f>IF(C16="NOT BAN","",_xlfn.XLOOKUP(A16,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F16" t="s">
+        <v>131</v>
+      </c>
+      <c r="G16" s="7">
+        <f>_xlfn.XLOOKUP(A16,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>5.1020408163265302E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
+        <v>42971568</v>
+      </c>
+      <c r="B17" s="5">
+        <v>46226.351898148147</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D17" t="e">
+        <f>IF(C17="NOT BAN","",_xlfn.XLOOKUP(A17,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E17" s="6" t="e">
+        <f>IF(C17="NOT BAN","",_xlfn.XLOOKUP(A17,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F17" t="s">
+        <v>130</v>
+      </c>
+      <c r="G17" s="7">
+        <f>_xlfn.XLOOKUP(A17,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>1.5151515151515152E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
+        <v>42997602</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46227.310555555552</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D18" t="e">
+        <f>IF(C18="NOT BAN","",_xlfn.XLOOKUP(A18,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E18" s="6" t="e">
+        <f>IF(C18="NOT BAN","",_xlfn.XLOOKUP(A18,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F18" t="s">
+        <v>130</v>
+      </c>
+      <c r="G18" s="7">
+        <f>_xlfn.XLOOKUP(A18,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>5.076142131979695E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
+        <v>43022614</v>
+      </c>
+      <c r="B19" s="5">
+        <v>46227.953402777777</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D19" t="e">
+        <f>IF(C19="NOT BAN","",_xlfn.XLOOKUP(A19,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E19" s="6" t="e">
+        <f>IF(C19="NOT BAN","",_xlfn.XLOOKUP(A19,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F19" t="s">
+        <v>130</v>
+      </c>
+      <c r="G19" s="7">
+        <f>_xlfn.XLOOKUP(A19,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>6.0606060606060606E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
+        <v>43081554</v>
+      </c>
+      <c r="B20" s="5">
+        <v>46230.316782407404</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D20" t="e">
+        <f>IF(C20="NOT BAN","",_xlfn.XLOOKUP(A20,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E20" s="6" t="e">
+        <f>IF(C20="NOT BAN","",_xlfn.XLOOKUP(A20,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F20" t="s">
+        <v>130</v>
+      </c>
+      <c r="G20" s="7">
+        <f>_xlfn.XLOOKUP(A20,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>7.462686567164179E-3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
+        <v>43110506</v>
+      </c>
+      <c r="B21" s="5">
+        <v>46231.34375</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D21" t="str">
+        <f>IF(C21="NOT BAN","",_xlfn.XLOOKUP(A21,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v/>
+      </c>
+      <c r="E21" s="6" t="str">
+        <f>IF(C21="NOT BAN","",_xlfn.XLOOKUP(A21,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v/>
+      </c>
+      <c r="F21" t="s">
+        <v>130</v>
+      </c>
+      <c r="G21" s="7">
+        <f>_xlfn.XLOOKUP(A21,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>8.4033613445378148E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
+        <v>43138108</v>
+      </c>
+      <c r="B22" s="5">
+        <v>46232.319733796299</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D22" t="e">
+        <f>IF(C22="NOT BAN","",_xlfn.XLOOKUP(A22,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E22" s="6" t="e">
+        <f>IF(C22="NOT BAN","",_xlfn.XLOOKUP(A22,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F22" t="s">
+        <v>130</v>
+      </c>
+      <c r="G22" s="7">
+        <f>_xlfn.XLOOKUP(A22,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
+        <v>43166702</v>
+      </c>
+      <c r="B23" s="5">
+        <v>46233.295995370368</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D23" t="e">
+        <f>IF(C23="NOT BAN","",_xlfn.XLOOKUP(A23,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E23" s="6" t="e">
+        <f>IF(C23="NOT BAN","",_xlfn.XLOOKUP(A23,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F23" t="s">
+        <v>130</v>
+      </c>
+      <c r="G23" s="7">
+        <f>_xlfn.XLOOKUP(A23,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>5.9523809523809521E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
+        <v>8200826</v>
+      </c>
+      <c r="B24" s="5">
+        <v>43951.628587962965</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D24" t="str">
+        <f>IF(C24="NOT BAN","",_xlfn.XLOOKUP(A24,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v/>
+      </c>
+      <c r="E24" s="6" t="str">
+        <f>IF(C24="NOT BAN","",_xlfn.XLOOKUP(A24,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v/>
+      </c>
+      <c r="F24" t="s">
+        <v>131</v>
+      </c>
+      <c r="G24" s="7">
+        <f>_xlfn.XLOOKUP(A24,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0.19748610103940054</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
+        <v>43230061</v>
+      </c>
+      <c r="B25" s="5">
+        <v>46235.320451388892</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D25" t="e">
+        <f>IF(C25="NOT BAN","",_xlfn.XLOOKUP(A25,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E25" s="6" t="e">
+        <f>IF(C25="NOT BAN","",_xlfn.XLOOKUP(A25,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F25" t="s">
+        <v>130</v>
+      </c>
+      <c r="G25" s="7">
+        <f>_xlfn.XLOOKUP(A25,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
+        <v>43290314</v>
+      </c>
+      <c r="B26" s="5">
+        <v>46237.319421296299</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D26" t="e">
+        <f>IF(C26="NOT BAN","",_xlfn.XLOOKUP(A26,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E26" s="6" t="e">
+        <f>IF(C26="NOT BAN","",_xlfn.XLOOKUP(A26,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F26" t="s">
+        <v>130</v>
+      </c>
+      <c r="G26" s="7">
+        <f>_xlfn.XLOOKUP(A26,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>7.5187969924812026E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
+        <v>43319297</v>
+      </c>
+      <c r="B27" s="5">
+        <v>46238.332465277781</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D27" t="e">
+        <f>IF(C27="NOT BAN","",_xlfn.XLOOKUP(A27,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E27" s="6" t="e">
+        <f>IF(C27="NOT BAN","",_xlfn.XLOOKUP(A27,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F27" t="s">
+        <v>130</v>
+      </c>
+      <c r="G27" s="7">
+        <f>_xlfn.XLOOKUP(A27,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
+        <v>43346700</v>
+      </c>
+      <c r="B28" s="5">
+        <v>46239.324108796296</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D28" t="e">
+        <f>IF(C28="NOT BAN","",_xlfn.XLOOKUP(A28,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E28" s="6" t="e">
+        <f>IF(C28="NOT BAN","",_xlfn.XLOOKUP(A28,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F28" t="s">
+        <v>130</v>
+      </c>
+      <c r="G28" s="7">
+        <f>_xlfn.XLOOKUP(A28,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
+        <v>43374604</v>
+      </c>
+      <c r="B29" s="5">
+        <v>46240.339444444442</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D29" t="e">
+        <f>IF(C29="NOT BAN","",_xlfn.XLOOKUP(A29,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E29" s="6" t="e">
+        <f>IF(C29="NOT BAN","",_xlfn.XLOOKUP(A29,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F29" t="s">
+        <v>130</v>
+      </c>
+      <c r="G29" s="7">
+        <f>_xlfn.XLOOKUP(A29,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
+        <v>43402439</v>
+      </c>
+      <c r="B30" s="5">
+        <v>46241.331238425926</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D30" t="e">
+        <f>IF(C30="NOT BAN","",_xlfn.XLOOKUP(A30,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E30" s="6" t="e">
+        <f>IF(C30="NOT BAN","",_xlfn.XLOOKUP(A30,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F30" t="s">
+        <v>130</v>
+      </c>
+      <c r="G30" s="7">
+        <f>_xlfn.XLOOKUP(A30,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>3.8461538461538464E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
+        <v>43430885</v>
+      </c>
+      <c r="B31" s="5">
+        <v>46242.334328703706</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D31" t="e">
+        <f>IF(C31="NOT BAN","",_xlfn.XLOOKUP(A31,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E31" s="6" t="e">
+        <f>IF(C31="NOT BAN","",_xlfn.XLOOKUP(A31,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F31" t="s">
+        <v>130</v>
+      </c>
+      <c r="G31" s="7">
+        <f>_xlfn.XLOOKUP(A31,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
+        <v>43539274</v>
+      </c>
+      <c r="B32" s="5">
+        <v>46246.331296296295</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D32" t="e">
+        <f>IF(C32="NOT BAN","",_xlfn.XLOOKUP(A32,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E32" s="6" t="e">
+        <f>IF(C32="NOT BAN","",_xlfn.XLOOKUP(A32,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F32" t="s">
+        <v>130</v>
+      </c>
+      <c r="G32" s="7">
+        <f>_xlfn.XLOOKUP(A32,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
+        <v>43566043</v>
+      </c>
+      <c r="B33" s="5">
+        <v>46247.329143518517</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D33" t="e">
+        <f>IF(C33="NOT BAN","",_xlfn.XLOOKUP(A33,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E33" s="6" t="e">
+        <f>IF(C33="NOT BAN","",_xlfn.XLOOKUP(A33,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F33" t="s">
+        <v>130</v>
+      </c>
+      <c r="G33" s="7">
+        <f>_xlfn.XLOOKUP(A33,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>7.1428571428571426E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
+        <v>43593087</v>
+      </c>
+      <c r="B34" s="5">
+        <v>46248.336215277777</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D34" t="e">
+        <f>IF(C34="NOT BAN","",_xlfn.XLOOKUP(A34,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E34" s="6" t="e">
+        <f>IF(C34="NOT BAN","",_xlfn.XLOOKUP(A34,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F34" t="s">
+        <v>130</v>
+      </c>
+      <c r="G34" s="7">
+        <f>_xlfn.XLOOKUP(A34,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="3">
+        <v>43614456</v>
+      </c>
+      <c r="B35" s="5">
+        <v>46248.851631944446</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D35" t="e">
+        <f>IF(C35="NOT BAN","",_xlfn.XLOOKUP(A35,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E35" s="6" t="e">
+        <f>IF(C35="NOT BAN","",_xlfn.XLOOKUP(A35,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F35" t="s">
+        <v>130</v>
+      </c>
+      <c r="G35" s="7">
+        <f>_xlfn.XLOOKUP(A35,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>1.0638297872340425E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <v>43674483</v>
+      </c>
+      <c r="B36" s="5">
+        <v>46251.327719907407</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D36" t="e">
+        <f>IF(C36="NOT BAN","",_xlfn.XLOOKUP(A36,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E36" s="6" t="e">
+        <f>IF(C36="NOT BAN","",_xlfn.XLOOKUP(A36,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F36" t="s">
+        <v>130</v>
+      </c>
+      <c r="G36" s="7">
+        <f>_xlfn.XLOOKUP(A36,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>9.9009900990099011E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <v>43862968</v>
+      </c>
+      <c r="B37" s="5">
+        <v>46258.331458333334</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D37" t="e">
+        <f>IF(C37="NOT BAN","",_xlfn.XLOOKUP(A37,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E37" s="6" t="e">
+        <f>IF(C37="NOT BAN","",_xlfn.XLOOKUP(A37,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F37" t="s">
+        <v>130</v>
+      </c>
+      <c r="G37" s="7">
+        <f>_xlfn.XLOOKUP(A37,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>6.9444444444444441E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>43891958</v>
+      </c>
+      <c r="B38" s="5">
+        <v>46259.325914351852</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D38" t="e">
+        <f>IF(C38="NOT BAN","",_xlfn.XLOOKUP(A38,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E38" s="6" t="e">
+        <f>IF(C38="NOT BAN","",_xlfn.XLOOKUP(A38,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F38" t="s">
+        <v>130</v>
+      </c>
+      <c r="G38" s="7">
+        <f>_xlfn.XLOOKUP(A38,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>8.2644628099173556E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
+        <v>43920615</v>
+      </c>
+      <c r="B39" s="5">
+        <v>46260.329965277779</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D39" t="e">
+        <f>IF(C39="NOT BAN","",_xlfn.XLOOKUP(A39,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E39" s="6" t="e">
+        <f>IF(C39="NOT BAN","",_xlfn.XLOOKUP(A39,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F39" t="s">
+        <v>130</v>
+      </c>
+      <c r="G39" s="7">
+        <f>_xlfn.XLOOKUP(A39,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="3">
+        <v>43949404</v>
+      </c>
+      <c r="B40" s="5">
+        <v>46261.33803240741</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D40" t="e">
+        <f>IF(C40="NOT BAN","",_xlfn.XLOOKUP(A40,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E40" s="6" t="e">
+        <f>IF(C40="NOT BAN","",_xlfn.XLOOKUP(A40,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F40" t="s">
+        <v>130</v>
+      </c>
+      <c r="G40" s="7">
+        <f>_xlfn.XLOOKUP(A40,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="3">
+        <v>43978801</v>
+      </c>
+      <c r="B41" s="5">
+        <v>46262.335601851853</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D41" t="e">
+        <f>IF(C41="NOT BAN","",_xlfn.XLOOKUP(A41,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E41" s="6" t="e">
+        <f>IF(C41="NOT BAN","",_xlfn.XLOOKUP(A41,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F41" t="s">
+        <v>130</v>
+      </c>
+      <c r="G41" s="7">
+        <f>_xlfn.XLOOKUP(A41,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
+        <v>44010401</v>
+      </c>
+      <c r="B42" s="5">
+        <v>46263.330763888887</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D42" t="e">
+        <f>IF(C42="NOT BAN","",_xlfn.XLOOKUP(A42,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$G$2:$G$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E42" s="6" t="e">
+        <f>IF(C42="NOT BAN","",_xlfn.XLOOKUP(A42,'[1]Results export'!$F$2:$F$33,'[1]Results export'!$C$2:$C$33))</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F42" t="s">
+        <v>130</v>
+      </c>
+      <c r="G42" s="7">
+        <f>_xlfn.XLOOKUP(A42,'[2]Results export'!$A$2:$A$42,'[2]Results export'!$R$2:$R$42)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G42" xr:uid="{DB011E51-5698-4F7F-B1C8-99B7D0DBCADD}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B917C4BF-6827-4C36-8E4A-9DB98CA460B6}">
   <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3834,7 +5743,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D93C4E66-FBE9-4925-8D98-3112F0EA52DB}">
   <dimension ref="A1:O20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4800,623 +6709,779 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4719527-41BF-4F40-B12E-62783B3C5FD2}">
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="8.88671875" style="1"/>
-    <col min="6" max="6" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.88671875" style="1"/>
+    <col min="7" max="7" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>8200826</v>
+      </c>
+      <c r="B2" s="1">
         <v>36425882</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>42406507</v>
+      </c>
+      <c r="B3" s="1">
         <v>2542992</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>42406507</v>
+      </c>
+      <c r="B4" s="1">
         <v>3158809</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>42406507</v>
+      </c>
+      <c r="B5" s="1">
         <v>3281810</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E5" s="1">
-        <f>COUNTA(C2:C52)</f>
+      <c r="F5" s="1">
+        <f>COUNTA(D2:D52)</f>
         <v>51</v>
       </c>
-      <c r="F5" s="1">
-        <f>COUNTIF(C2:C52,F4)</f>
+      <c r="G5" s="1">
+        <f>COUNTIF(D2:D52,G4)</f>
         <v>29</v>
       </c>
-      <c r="G5" s="1">
-        <f>COUNTIF(C2:C52,G4)</f>
+      <c r="H5" s="1">
+        <f>COUNTIF(D2:D52,H4)</f>
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>42406507</v>
+      </c>
+      <c r="B6" s="1">
         <v>3415189</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="F6" s="2">
-        <f>F5/E5</f>
+      <c r="G6" s="2">
+        <f>G5/F5</f>
         <v>0.56862745098039214</v>
       </c>
-      <c r="G6" s="2">
-        <f>G5/E5</f>
+      <c r="H6" s="2">
+        <f>H5/F5</f>
         <v>0.43137254901960786</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>42406507</v>
+      </c>
+      <c r="B7" s="1">
         <v>3434386</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>42406507</v>
+      </c>
+      <c r="B8" s="1">
         <v>3531594</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>42406507</v>
+      </c>
+      <c r="B9" s="1">
         <v>3819032</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>42406507</v>
+      </c>
+      <c r="B10" s="1">
         <v>4167618</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="D10" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>42406507</v>
+      </c>
+      <c r="B11" s="1">
         <v>4179701</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>42406507</v>
+      </c>
+      <c r="B12" s="1">
         <v>4188518</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>42406507</v>
+      </c>
+      <c r="B13" s="1">
         <v>4253659</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>42406507</v>
+      </c>
+      <c r="B14" s="1">
         <v>4276951</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="1">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>42406507</v>
+      </c>
+      <c r="B15" s="1">
         <v>4726514</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="1">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>42406507</v>
+      </c>
+      <c r="B16" s="1">
         <v>42011766</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="1">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>42406507</v>
+      </c>
+      <c r="B17" s="1">
         <v>42011817</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="D17" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="1">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>42406507</v>
+      </c>
+      <c r="B18" s="1">
         <v>42012426</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="1">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>42406507</v>
+      </c>
+      <c r="B19" s="1">
         <v>42077631</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="1">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>42406507</v>
+      </c>
+      <c r="B20" s="1">
         <v>42426592</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="1">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>42406507</v>
+      </c>
+      <c r="B21" s="1">
         <v>42426641</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="1">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>42406507</v>
+      </c>
+      <c r="B22" s="1">
         <v>42758642</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="D22" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="1">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>42406507</v>
+      </c>
+      <c r="B23" s="1">
         <v>42787717</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="1">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>42426592</v>
+      </c>
+      <c r="B24" s="1">
         <v>42406507</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="1">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>42426641</v>
+      </c>
+      <c r="B25" s="1">
         <v>42598944</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="C25" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="1">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>42458992</v>
+      </c>
+      <c r="B26" s="1">
         <v>42459099</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="D26" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="1">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>42458992</v>
+      </c>
+      <c r="B27" s="1">
         <v>42459206</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="1">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>42458992</v>
+      </c>
+      <c r="B28" s="1">
         <v>42459241</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="D28" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="1">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>42458992</v>
+      </c>
+      <c r="B29" s="1">
         <v>42459298</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="C29" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="D29" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="1">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>42459041</v>
+      </c>
+      <c r="B30" s="1">
         <v>42458992</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="C30" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="D30" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="1">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>42459041</v>
+      </c>
+      <c r="B31" s="1">
         <v>42459148</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="1">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>42731028</v>
+      </c>
+      <c r="B32" s="1">
         <v>42705635</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="C32" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="1">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>42997602</v>
+      </c>
+      <c r="B33" s="1">
         <v>43022302</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="C33" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="1">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>42997602</v>
+      </c>
+      <c r="B34" s="1">
         <v>43022440</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="C34" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="1">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>43346700</v>
+      </c>
+      <c r="B35" s="1">
         <v>43375656</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="C35" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="1">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>8200826</v>
+      </c>
+      <c r="B36" s="1">
         <v>16372934</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="C36" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="D36" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="1">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>42406507</v>
+      </c>
+      <c r="B37" s="1">
         <v>3463245</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="C37" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="D37" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="1">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>42406507</v>
+      </c>
+      <c r="B38" s="1">
         <v>3711577</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="C38" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="D38" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="1">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>42406507</v>
+      </c>
+      <c r="B39" s="1">
         <v>3728922</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="C39" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="D39" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="1">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>42406507</v>
+      </c>
+      <c r="B40" s="1">
         <v>3754003</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="D40" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="1">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>42406507</v>
+      </c>
+      <c r="B41" s="1">
         <v>4239307</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="C41" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="D41" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="1">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>42406507</v>
+      </c>
+      <c r="B42" s="1">
         <v>31956677</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="C42" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="1">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>42406507</v>
+      </c>
+      <c r="B43" s="1">
         <v>42010347</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="C43" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="D43" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="1">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>42406507</v>
+      </c>
+      <c r="B44" s="1">
         <v>42012522</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="C44" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="D44" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="1">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>42406507</v>
+      </c>
+      <c r="B45" s="1">
         <v>42079879</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="C45" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="D45" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="1">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>42406507</v>
+      </c>
+      <c r="B46" s="1">
         <v>42814075</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="C46" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="D46" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="1">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>42406507</v>
+      </c>
+      <c r="B47" s="1">
         <v>43110281</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="C47" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="1">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>42458992</v>
+      </c>
+      <c r="B48" s="1">
         <v>42459041</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="C48" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C48" s="1" t="s">
+      <c r="D48" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="1">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>42463024</v>
+      </c>
+      <c r="B49" s="1">
         <v>42463063</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="C49" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C49" s="1" t="s">
+      <c r="D49" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="1">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>42463063</v>
+      </c>
+      <c r="B50" s="1">
         <v>42463024</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="C50" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="D50" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="1">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>42705635</v>
+      </c>
+      <c r="B51" s="1">
         <v>42731028</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="C51" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="D51" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="1">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>43593087</v>
+      </c>
+      <c r="B52" s="1">
         <v>43613297</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="C52" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="D52" s="1" t="s">
         <v>113</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C52" xr:uid="{25ED12FD-7613-4161-AB77-60A5E5F0FD4C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>